<commit_message>
30.04. Data and Config Update
</commit_message>
<xml_diff>
--- a/testdata/data.xlsx
+++ b/testdata/data.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000"/>
+    <workbookView windowWidth="28800" windowHeight="12240"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -291,17 +291,17 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF800080"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
     </font>
     <font>
       <u/>
@@ -769,7 +769,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
@@ -909,14 +909,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="6" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="6" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" quotePrefix="1">
       <alignment vertical="center"/>
@@ -934,7 +934,7 @@
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
     <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
     <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
     <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
     <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
@@ -1593,7 +1593,7 @@
       <c r="AD1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="6" t="s">
+      <c r="AE1" s="4" t="s">
         <v>30</v>
       </c>
       <c r="AF1" s="1" t="s">
@@ -1646,7 +1646,7 @@
       </c>
     </row>
     <row r="2" s="2" customFormat="1" spans="1:47">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="5" t="s">
         <v>46</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -1664,7 +1664,7 @@
       <c r="F2" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="G2" s="6" t="s">
         <v>51</v>
       </c>
       <c r="H2" s="2" t="s">
@@ -1789,7 +1789,7 @@
       </c>
     </row>
     <row r="3" s="2" customFormat="1" spans="1:47">
-      <c r="A3" s="4" t="s">
+      <c r="A3" s="5" t="s">
         <v>46</v>
       </c>
       <c r="B3" s="2" t="s">
@@ -1807,7 +1807,7 @@
       <c r="F3" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G3" s="5" t="s">
+      <c r="G3" s="6" t="s">
         <v>51</v>
       </c>
       <c r="H3" s="2" t="s">
@@ -1932,7 +1932,7 @@
       </c>
     </row>
     <row r="4" s="2" customFormat="1" spans="1:47">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="5" t="s">
         <v>46</v>
       </c>
       <c r="B4" s="2" t="s">
@@ -1950,7 +1950,7 @@
       <c r="F4" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G4" s="5" t="s">
+      <c r="G4" s="6" t="s">
         <v>51</v>
       </c>
       <c r="H4" s="2" t="s">
@@ -2075,7 +2075,7 @@
       </c>
     </row>
     <row r="5" s="2" customFormat="1" spans="1:47">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="5" t="s">
         <v>46</v>
       </c>
       <c r="B5" s="2" t="s">
@@ -2093,7 +2093,7 @@
       <c r="F5" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="6" t="s">
         <v>51</v>
       </c>
       <c r="H5" s="2" t="s">
@@ -2218,7 +2218,7 @@
       </c>
     </row>
     <row r="6" s="2" customFormat="1" spans="1:47">
-      <c r="A6" s="4" t="s">
+      <c r="A6" s="5" t="s">
         <v>46</v>
       </c>
       <c r="B6" s="2" t="s">
@@ -2236,7 +2236,7 @@
       <c r="F6" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G6" s="5" t="s">
+      <c r="G6" s="6" t="s">
         <v>51</v>
       </c>
       <c r="H6" s="2" t="s">
@@ -2361,7 +2361,7 @@
       </c>
     </row>
     <row r="7" s="2" customFormat="1" spans="1:47">
-      <c r="A7" s="4" t="s">
+      <c r="A7" s="5" t="s">
         <v>46</v>
       </c>
       <c r="B7" s="2" t="s">
@@ -2379,7 +2379,7 @@
       <c r="F7" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="G7" s="6" t="s">
         <v>51</v>
       </c>
       <c r="H7" s="2" t="s">
@@ -2504,7 +2504,7 @@
       </c>
     </row>
     <row r="8" s="2" customFormat="1" spans="1:47">
-      <c r="A8" s="4" t="s">
+      <c r="A8" s="5" t="s">
         <v>46</v>
       </c>
       <c r="B8" s="2" t="s">
@@ -2522,7 +2522,7 @@
       <c r="F8" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="G8" s="5" t="s">
+      <c r="G8" s="6" t="s">
         <v>51</v>
       </c>
       <c r="H8" s="2" t="s">

</xml_diff>

<commit_message>
14.05. Moj komp pred regresiju na drugom kompu
</commit_message>
<xml_diff>
--- a/testdata/data.xlsx
+++ b/testdata/data.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="8400"/>
+    <workbookView windowWidth="23040" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="125">
   <si>
     <t>username</t>
   </si>
@@ -266,6 +266,9 @@
     <t>Enil ČIĆVI</t>
   </si>
   <si>
+    <t>ČIĆVI OLIK</t>
+  </si>
+  <si>
     <t>205-9001015647000-10</t>
   </si>
   <si>
@@ -323,46 +326,49 @@
     <t>205-9001007839862-95</t>
   </si>
   <si>
+    <t>Mastercard Installment Card</t>
+  </si>
+  <si>
+    <t>5309 **** **** 0724</t>
+  </si>
+  <si>
+    <t>4313********5507</t>
+  </si>
+  <si>
+    <t>4313 **** **** 5507</t>
+  </si>
+  <si>
+    <t>9011004938920</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> A vista depozitni račun </t>
+  </si>
+  <si>
+    <t>9011008661345</t>
+  </si>
+  <si>
+    <t>9032005130761</t>
+  </si>
+  <si>
+    <t>9032005664316</t>
+  </si>
+  <si>
+    <t>0049015018282</t>
+  </si>
+  <si>
+    <t>0049038646620</t>
+  </si>
+  <si>
+    <t>Jail ĆEVGIMILĆ</t>
+  </si>
+  <si>
+    <t>205-9001007668260-25</t>
+  </si>
+  <si>
+    <t>RS35 2059 0310 0108 6257 79</t>
+  </si>
+  <si>
     <t>Visa Gold revolving</t>
-  </si>
-  <si>
-    <t>4176 **** **** 4784</t>
-  </si>
-  <si>
-    <t>4313********5507</t>
-  </si>
-  <si>
-    <t>4313 **** **** 5507</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> A vista depozitni račun </t>
-  </si>
-  <si>
-    <t>9011004938920</t>
-  </si>
-  <si>
-    <t>9011008661345</t>
-  </si>
-  <si>
-    <t>9032005130761</t>
-  </si>
-  <si>
-    <t>9032005664316</t>
-  </si>
-  <si>
-    <t>0049015018282</t>
-  </si>
-  <si>
-    <t>0049038646620</t>
-  </si>
-  <si>
-    <t>Jail ĆEVGIMILĆ</t>
-  </si>
-  <si>
-    <t>205-9001007668260-25</t>
-  </si>
-  <si>
-    <t>RS35 2059 0310 0108 6257 79</t>
   </si>
   <si>
     <t>4176 **** **** 4328</t>
@@ -1622,7 +1628,7 @@
     <col min="13" max="13" width="24.2222222222222" style="3" customWidth="1"/>
     <col min="14" max="14" width="27.8888888888889" style="3" customWidth="1"/>
     <col min="15" max="15" width="28.8611111111111" style="3" customWidth="1"/>
-    <col min="16" max="16" width="24.2222222222222" style="3" customWidth="1"/>
+    <col min="16" max="16" width="26.6666666666667" style="3" customWidth="1"/>
     <col min="17" max="17" width="23.6666666666667" style="3" customWidth="1"/>
     <col min="18" max="18" width="31.2222222222222" style="3" customWidth="1"/>
     <col min="19" max="19" width="19.5555555555556" style="3" customWidth="1"/>
@@ -1954,7 +1960,7 @@
         <v>48</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>52</v>
+        <v>79</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>52</v>
@@ -1963,19 +1969,19 @@
         <v>51</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="J3" s="2" t="s">
         <v>54</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="M3" s="2" t="s">
         <v>54</v>
@@ -1984,7 +1990,7 @@
         <v>52</v>
       </c>
       <c r="O3" s="7" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="P3" s="2" t="s">
         <v>52</v>
@@ -2023,7 +2029,7 @@
         <v>67</v>
       </c>
       <c r="AB3" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="AC3" s="2" t="s">
         <v>52</v>
@@ -2050,12 +2056,12 @@
         <v>52</v>
       </c>
       <c r="AK3" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" s="3" customFormat="1" spans="1:47">
       <c r="A4" s="1" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>52</v>
@@ -2076,28 +2082,28 @@
         <v>54</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>51</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="M4" s="2" t="s">
         <v>51</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="O4" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="P4" s="2" t="s">
         <v>52</v>
@@ -2163,12 +2169,12 @@
         <v>52</v>
       </c>
       <c r="AK4" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5" s="2" customFormat="1" ht="15" customHeight="1" spans="1:47">
       <c r="A5" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>52</v>
@@ -2180,25 +2186,25 @@
         <v>48</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="G5" s="8" t="s">
         <v>51</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>54</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L5" s="2" t="s">
         <v>52</v>
@@ -2213,19 +2219,19 @@
         <v>52</v>
       </c>
       <c r="P5" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="R5" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="S5" s="2" t="s">
         <v>58</v>
       </c>
       <c r="T5" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="U5" s="2" t="s">
         <v>52</v>
@@ -2234,28 +2240,28 @@
         <v>52</v>
       </c>
       <c r="W5" s="2" t="s">
-        <v>102</v>
+        <v>63</v>
       </c>
       <c r="X5" s="11" t="s">
         <v>103</v>
       </c>
       <c r="Y5" s="2" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="Z5" s="11" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="AA5" s="2" t="s">
         <v>67</v>
       </c>
       <c r="AB5" s="11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="AC5" s="2" t="s">
         <v>67</v>
       </c>
       <c r="AD5" s="11" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="AE5" s="2" t="s">
         <v>52</v>
@@ -2267,13 +2273,13 @@
         <v>70</v>
       </c>
       <c r="AH5" s="11" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="AI5" s="9" t="s">
         <v>70</v>
       </c>
       <c r="AJ5" s="11" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="AK5" s="2" t="s">
         <v>55</v>
@@ -2281,7 +2287,7 @@
     </row>
     <row r="6" s="3" customFormat="1" ht="13" customHeight="1" spans="1:47">
       <c r="A6" s="10" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>52</v>
@@ -2302,7 +2308,7 @@
         <v>54</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>52</v>
@@ -2311,10 +2317,10 @@
         <v>51</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="L6" s="5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="M6" s="2" t="s">
         <v>52</v>
@@ -2326,19 +2332,19 @@
         <v>52</v>
       </c>
       <c r="P6" s="2" t="s">
-        <v>98</v>
+        <v>113</v>
       </c>
       <c r="Q6" s="2" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="R6" s="2" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="S6" s="2" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="T6" s="2" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="U6" s="2" t="s">
         <v>52</v>
@@ -2380,13 +2386,13 @@
         <v>70</v>
       </c>
       <c r="AH6" s="12" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AI6" s="9" t="s">
         <v>70</v>
       </c>
       <c r="AJ6" s="12" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="AK6" s="2" t="s">
         <v>55</v>
@@ -2394,7 +2400,7 @@
     </row>
     <row r="7" s="3" customFormat="1" spans="1:47">
       <c r="A7" s="10" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>52</v>
@@ -2415,7 +2421,7 @@
         <v>54</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>52</v>
@@ -2427,7 +2433,7 @@
         <v>52</v>
       </c>
       <c r="L7" s="5" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="M7" s="2" t="s">
         <v>52</v>
@@ -2507,7 +2513,7 @@
     </row>
     <row r="8" spans="1:47">
       <c r="A8" s="10" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>52</v>
@@ -2561,10 +2567,10 @@
         <v>52</v>
       </c>
       <c r="S8" s="3" t="s">
-        <v>98</v>
+        <v>113</v>
       </c>
       <c r="T8" s="3" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="U8" s="3" t="s">
         <v>52</v>

</xml_diff>

<commit_message>
15.05. Posle velike regresije sa drugog kompa
</commit_message>
<xml_diff>
--- a/testdata/data.xlsx
+++ b/testdata/data.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000"/>
+    <workbookView windowWidth="20490" windowHeight="7500"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="126">
   <si>
     <t>username</t>
   </si>
@@ -381,6 +381,9 @@
   </si>
   <si>
     <t>6556 **** **** 1233</t>
+  </si>
+  <si>
+    <t>Stambeni kredit</t>
   </si>
   <si>
     <t>0049005001233</t>
@@ -424,6 +427,7 @@
     </font>
     <font>
       <sz val="11"/>
+      <color rgb="FF1E1E1E"/>
       <name val="Calibri"/>
       <charset val="134"/>
     </font>
@@ -435,7 +439,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF1E1E1E"/>
       <name val="Calibri"/>
       <charset val="134"/>
     </font>
@@ -1053,25 +1056,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" quotePrefix="1">
@@ -1093,7 +1096,7 @@
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
     <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
     <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
     <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
     <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
@@ -1614,50 +1617,50 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:AU13"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="17.712962962963" style="3" customWidth="1"/>
-    <col min="2" max="2" width="33.5740740740741" style="3" customWidth="1"/>
-    <col min="3" max="3" width="8.88888888888889" style="3"/>
-    <col min="4" max="6" width="22.1111111111111" style="3" customWidth="1"/>
+    <col min="1" max="1" width="17.7142857142857" style="3" customWidth="1"/>
+    <col min="2" max="2" width="33.5714285714286" style="3" customWidth="1"/>
+    <col min="3" max="3" width="8.88571428571429" style="3"/>
+    <col min="4" max="6" width="22.1142857142857" style="3" customWidth="1"/>
     <col min="7" max="7" width="33" style="3" customWidth="1"/>
     <col min="8" max="8" width="23.6666666666667" style="3" customWidth="1"/>
-    <col min="9" max="10" width="33.8888888888889" style="3" customWidth="1"/>
+    <col min="9" max="10" width="33.8857142857143" style="3" customWidth="1"/>
     <col min="11" max="11" width="23.6666666666667" style="3" customWidth="1"/>
-    <col min="12" max="12" width="28.7407407407407" style="3" customWidth="1"/>
-    <col min="13" max="13" width="24.2222222222222" style="3" customWidth="1"/>
-    <col min="14" max="14" width="27.8888888888889" style="3" customWidth="1"/>
-    <col min="15" max="15" width="28.8611111111111" style="3" customWidth="1"/>
+    <col min="12" max="12" width="28.7428571428571" style="3" customWidth="1"/>
+    <col min="13" max="13" width="24.2190476190476" style="3" customWidth="1"/>
+    <col min="14" max="14" width="27.8857142857143" style="3" customWidth="1"/>
+    <col min="15" max="15" width="28.8571428571429" style="3" customWidth="1"/>
     <col min="16" max="16" width="26.6666666666667" style="3" customWidth="1"/>
     <col min="17" max="17" width="23.6666666666667" style="3" customWidth="1"/>
-    <col min="18" max="18" width="31.2222222222222" style="3" customWidth="1"/>
-    <col min="19" max="19" width="19.5555555555556" style="3" customWidth="1"/>
-    <col min="20" max="20" width="21.4444444444444" style="3" customWidth="1"/>
-    <col min="21" max="23" width="24.1111111111111" style="3" customWidth="1"/>
-    <col min="24" max="24" width="25.4259259259259" style="3" customWidth="1"/>
-    <col min="25" max="25" width="24.1111111111111" style="3" customWidth="1"/>
-    <col min="26" max="26" width="25.8796296296296" style="3" customWidth="1"/>
-    <col min="27" max="27" width="24.1111111111111" style="3" customWidth="1"/>
-    <col min="28" max="28" width="32.1851851851852" style="3" customWidth="1"/>
-    <col min="29" max="29" width="21.4444444444444" style="3" customWidth="1"/>
+    <col min="18" max="18" width="31.2190476190476" style="3" customWidth="1"/>
+    <col min="19" max="19" width="19.552380952381" style="3" customWidth="1"/>
+    <col min="20" max="20" width="21.447619047619" style="3" customWidth="1"/>
+    <col min="21" max="23" width="24.1142857142857" style="3" customWidth="1"/>
+    <col min="24" max="24" width="25.4285714285714" style="3" customWidth="1"/>
+    <col min="25" max="25" width="24.1142857142857" style="3" customWidth="1"/>
+    <col min="26" max="26" width="25.8761904761905" style="3" customWidth="1"/>
+    <col min="27" max="27" width="24.1142857142857" style="3" customWidth="1"/>
+    <col min="28" max="28" width="32.1809523809524" style="3" customWidth="1"/>
+    <col min="29" max="29" width="21.447619047619" style="3" customWidth="1"/>
     <col min="30" max="30" width="32.6666666666667" style="3" customWidth="1"/>
     <col min="31" max="31" width="17.6666666666667" style="3" customWidth="1"/>
-    <col min="32" max="32" width="23.8888888888889" style="3" customWidth="1"/>
-    <col min="33" max="33" width="26.0092592592593" style="3" customWidth="1"/>
-    <col min="34" max="34" width="23.5555555555556" style="3" customWidth="1"/>
-    <col min="35" max="35" width="26.0092592592593" style="3" customWidth="1"/>
-    <col min="36" max="36" width="23.5555555555556" style="3" customWidth="1"/>
-    <col min="37" max="37" width="23.7777777777778" style="3" customWidth="1"/>
+    <col min="32" max="32" width="23.8857142857143" style="3" customWidth="1"/>
+    <col min="33" max="33" width="26.0095238095238" style="3" customWidth="1"/>
+    <col min="34" max="34" width="23.552380952381" style="3" customWidth="1"/>
+    <col min="35" max="35" width="26.0095238095238" style="3" customWidth="1"/>
+    <col min="36" max="36" width="23.552380952381" style="3" customWidth="1"/>
+    <col min="37" max="37" width="23.7809523809524" style="3" customWidth="1"/>
     <col min="38" max="38" width="31" style="3" customWidth="1"/>
-    <col min="39" max="40" width="32.8888888888889" style="3" customWidth="1"/>
-    <col min="41" max="41" width="29.1111111111111" style="3" customWidth="1"/>
+    <col min="39" max="40" width="32.8857142857143" style="3" customWidth="1"/>
+    <col min="41" max="41" width="29.1142857142857" style="3" customWidth="1"/>
     <col min="42" max="42" width="33" style="3" customWidth="1"/>
-    <col min="43" max="43" width="37.1111111111111" style="3" customWidth="1"/>
-    <col min="44" max="44" width="31.2222222222222" style="3" customWidth="1"/>
-    <col min="45" max="45" width="18.5555555555556" style="3" customWidth="1"/>
+    <col min="43" max="43" width="37.1142857142857" style="3" customWidth="1"/>
+    <col min="44" max="44" width="31.2190476190476" style="3" customWidth="1"/>
+    <col min="45" max="45" width="18.552380952381" style="3" customWidth="1"/>
     <col min="46" max="46" width="16.6666666666667" style="3" customWidth="1"/>
-    <col min="47" max="47" width="14.7777777777778" style="3" customWidth="1"/>
-    <col min="48" max="16384" width="8.88888888888889" style="3"/>
+    <col min="47" max="47" width="14.7809523809524" style="3" customWidth="1"/>
+    <col min="48" max="16384" width="8.88571428571429" style="3"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:47">
@@ -1754,7 +1757,7 @@
       <c r="AE1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="4" t="s">
+      <c r="AF1" s="9" t="s">
         <v>31</v>
       </c>
       <c r="AG1" s="1" t="s">
@@ -1825,7 +1828,7 @@
       <c r="G2" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" s="4" t="s">
         <v>52</v>
       </c>
       <c r="I2" s="2" t="s">
@@ -1946,7 +1949,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="3" s="3" customFormat="1" spans="1:47">
+    <row r="3" s="3" customFormat="1" spans="1:37">
       <c r="A3" s="1" t="s">
         <v>78</v>
       </c>
@@ -1971,7 +1974,7 @@
       <c r="H3" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="I3" s="7" t="s">
         <v>81</v>
       </c>
       <c r="J3" s="2" t="s">
@@ -1989,7 +1992,7 @@
       <c r="N3" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="O3" s="7" t="s">
+      <c r="O3" s="8" t="s">
         <v>84</v>
       </c>
       <c r="P3" s="2" t="s">
@@ -2059,7 +2062,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="4" s="3" customFormat="1" spans="1:47">
+    <row r="4" s="3" customFormat="1" spans="1:37">
       <c r="A4" s="1" t="s">
         <v>87</v>
       </c>
@@ -2172,7 +2175,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="5" s="2" customFormat="1" ht="15" customHeight="1" spans="1:47">
+    <row r="5" s="2" customFormat="1" customHeight="1" spans="1:37">
       <c r="A5" s="1" t="s">
         <v>93</v>
       </c>
@@ -2185,13 +2188,13 @@
       <c r="D5" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="F5" s="8" t="s">
+      <c r="F5" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="G5" s="5" t="s">
         <v>51</v>
       </c>
       <c r="H5" s="2" t="s">
@@ -2269,13 +2272,13 @@
       <c r="AF5" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="AG5" s="9" t="s">
+      <c r="AG5" s="10" t="s">
         <v>70</v>
       </c>
       <c r="AH5" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="AI5" s="9" t="s">
+      <c r="AI5" s="10" t="s">
         <v>70</v>
       </c>
       <c r="AJ5" s="11" t="s">
@@ -2285,8 +2288,8 @@
         <v>55</v>
       </c>
     </row>
-    <row r="6" s="3" customFormat="1" ht="13" customHeight="1" spans="1:47">
-      <c r="A6" s="10" t="s">
+    <row r="6" s="3" customFormat="1" ht="13" customHeight="1" spans="1:37">
+      <c r="A6" s="6" t="s">
         <v>110</v>
       </c>
       <c r="B6" s="3" t="s">
@@ -2319,7 +2322,7 @@
       <c r="K6" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="L6" s="5" t="s">
+      <c r="L6" s="4" t="s">
         <v>112</v>
       </c>
       <c r="M6" s="2" t="s">
@@ -2382,25 +2385,25 @@
       <c r="AF6" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="AG6" s="9" t="s">
+      <c r="AG6" s="10" t="s">
+        <v>118</v>
+      </c>
+      <c r="AH6" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="AI6" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="AH6" s="12" t="s">
-        <v>118</v>
-      </c>
-      <c r="AI6" s="9" t="s">
-        <v>70</v>
-      </c>
       <c r="AJ6" s="12" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="AK6" s="2" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="7" s="3" customFormat="1" spans="1:47">
-      <c r="A7" s="10" t="s">
-        <v>120</v>
+    <row r="7" s="3" customFormat="1" spans="1:37">
+      <c r="A7" s="6" t="s">
+        <v>121</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>52</v>
@@ -2421,7 +2424,7 @@
         <v>54</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>52</v>
@@ -2432,8 +2435,8 @@
       <c r="K7" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="L7" s="5" t="s">
-        <v>122</v>
+      <c r="L7" s="4" t="s">
+        <v>123</v>
       </c>
       <c r="M7" s="2" t="s">
         <v>52</v>
@@ -2512,8 +2515,8 @@
       </c>
     </row>
     <row r="8" spans="1:47">
-      <c r="A8" s="10" t="s">
-        <v>123</v>
+      <c r="A8" s="6" t="s">
+        <v>124</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>52</v>
@@ -2570,7 +2573,7 @@
         <v>113</v>
       </c>
       <c r="T8" s="3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="U8" s="3" t="s">
         <v>52</v>
@@ -2654,7 +2657,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="13" spans="1:47">
+    <row r="13" spans="11:11">
       <c r="K13" s="2"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
27.05. Moj komp pred regresiju na drugom kompu
</commit_message>
<xml_diff>
--- a/testdata/data.xlsx
+++ b/testdata/data.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7500"/>
+    <workbookView windowWidth="23040" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -242,7 +242,7 @@
     <t>Gotovinski kredit</t>
   </si>
   <si>
-    <t>0049005026910</t>
+    <t>0049018637013</t>
   </si>
   <si>
     <t>KOAR TGR</t>
@@ -427,7 +427,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF1E1E1E"/>
       <name val="Calibri"/>
       <charset val="134"/>
     </font>
@@ -439,6 +438,7 @@
     </font>
     <font>
       <sz val="11"/>
+      <color rgb="FF1E1E1E"/>
       <name val="Calibri"/>
       <charset val="134"/>
     </font>
@@ -1056,25 +1056,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" quotePrefix="1">
@@ -1096,7 +1096,7 @@
     <cellStyle name="Note" xfId="8" builtinId="10"/>
     <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
     <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
     <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
     <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
     <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
@@ -1617,50 +1617,50 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:AU13"/>
-  <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="17.7142857142857" style="3" customWidth="1"/>
-    <col min="2" max="2" width="33.5714285714286" style="3" customWidth="1"/>
-    <col min="3" max="3" width="8.88571428571429" style="3"/>
-    <col min="4" max="6" width="22.1142857142857" style="3" customWidth="1"/>
+    <col min="1" max="1" width="17.712962962963" style="3" customWidth="1"/>
+    <col min="2" max="2" width="33.5740740740741" style="3" customWidth="1"/>
+    <col min="3" max="3" width="8.88888888888889" style="3"/>
+    <col min="4" max="6" width="22.1111111111111" style="3" customWidth="1"/>
     <col min="7" max="7" width="33" style="3" customWidth="1"/>
     <col min="8" max="8" width="23.6666666666667" style="3" customWidth="1"/>
-    <col min="9" max="10" width="33.8857142857143" style="3" customWidth="1"/>
+    <col min="9" max="10" width="33.8888888888889" style="3" customWidth="1"/>
     <col min="11" max="11" width="23.6666666666667" style="3" customWidth="1"/>
-    <col min="12" max="12" width="28.7428571428571" style="3" customWidth="1"/>
-    <col min="13" max="13" width="24.2190476190476" style="3" customWidth="1"/>
-    <col min="14" max="14" width="27.8857142857143" style="3" customWidth="1"/>
-    <col min="15" max="15" width="28.8571428571429" style="3" customWidth="1"/>
+    <col min="12" max="12" width="28.7407407407407" style="3" customWidth="1"/>
+    <col min="13" max="13" width="24.2222222222222" style="3" customWidth="1"/>
+    <col min="14" max="14" width="27.8888888888889" style="3" customWidth="1"/>
+    <col min="15" max="15" width="28.8611111111111" style="3" customWidth="1"/>
     <col min="16" max="16" width="26.6666666666667" style="3" customWidth="1"/>
     <col min="17" max="17" width="23.6666666666667" style="3" customWidth="1"/>
-    <col min="18" max="18" width="31.2190476190476" style="3" customWidth="1"/>
-    <col min="19" max="19" width="19.552380952381" style="3" customWidth="1"/>
-    <col min="20" max="20" width="21.447619047619" style="3" customWidth="1"/>
-    <col min="21" max="23" width="24.1142857142857" style="3" customWidth="1"/>
-    <col min="24" max="24" width="25.4285714285714" style="3" customWidth="1"/>
-    <col min="25" max="25" width="24.1142857142857" style="3" customWidth="1"/>
-    <col min="26" max="26" width="25.8761904761905" style="3" customWidth="1"/>
-    <col min="27" max="27" width="24.1142857142857" style="3" customWidth="1"/>
-    <col min="28" max="28" width="32.1809523809524" style="3" customWidth="1"/>
-    <col min="29" max="29" width="21.447619047619" style="3" customWidth="1"/>
+    <col min="18" max="18" width="31.2222222222222" style="3" customWidth="1"/>
+    <col min="19" max="19" width="19.5555555555556" style="3" customWidth="1"/>
+    <col min="20" max="20" width="21.4444444444444" style="3" customWidth="1"/>
+    <col min="21" max="23" width="24.1111111111111" style="3" customWidth="1"/>
+    <col min="24" max="24" width="25.4259259259259" style="3" customWidth="1"/>
+    <col min="25" max="25" width="24.1111111111111" style="3" customWidth="1"/>
+    <col min="26" max="26" width="25.8796296296296" style="3" customWidth="1"/>
+    <col min="27" max="27" width="24.1111111111111" style="3" customWidth="1"/>
+    <col min="28" max="28" width="32.1851851851852" style="3" customWidth="1"/>
+    <col min="29" max="29" width="21.4444444444444" style="3" customWidth="1"/>
     <col min="30" max="30" width="32.6666666666667" style="3" customWidth="1"/>
     <col min="31" max="31" width="17.6666666666667" style="3" customWidth="1"/>
-    <col min="32" max="32" width="23.8857142857143" style="3" customWidth="1"/>
-    <col min="33" max="33" width="26.0095238095238" style="3" customWidth="1"/>
-    <col min="34" max="34" width="23.552380952381" style="3" customWidth="1"/>
-    <col min="35" max="35" width="26.0095238095238" style="3" customWidth="1"/>
-    <col min="36" max="36" width="23.552380952381" style="3" customWidth="1"/>
-    <col min="37" max="37" width="23.7809523809524" style="3" customWidth="1"/>
+    <col min="32" max="32" width="23.8888888888889" style="3" customWidth="1"/>
+    <col min="33" max="33" width="26.0092592592593" style="3" customWidth="1"/>
+    <col min="34" max="34" width="23.5555555555556" style="3" customWidth="1"/>
+    <col min="35" max="35" width="26.0092592592593" style="3" customWidth="1"/>
+    <col min="36" max="36" width="23.5555555555556" style="3" customWidth="1"/>
+    <col min="37" max="37" width="23.7777777777778" style="3" customWidth="1"/>
     <col min="38" max="38" width="31" style="3" customWidth="1"/>
-    <col min="39" max="40" width="32.8857142857143" style="3" customWidth="1"/>
-    <col min="41" max="41" width="29.1142857142857" style="3" customWidth="1"/>
+    <col min="39" max="40" width="32.8888888888889" style="3" customWidth="1"/>
+    <col min="41" max="41" width="29.1111111111111" style="3" customWidth="1"/>
     <col min="42" max="42" width="33" style="3" customWidth="1"/>
-    <col min="43" max="43" width="37.1142857142857" style="3" customWidth="1"/>
-    <col min="44" max="44" width="31.2190476190476" style="3" customWidth="1"/>
-    <col min="45" max="45" width="18.552380952381" style="3" customWidth="1"/>
+    <col min="43" max="43" width="37.1111111111111" style="3" customWidth="1"/>
+    <col min="44" max="44" width="31.2222222222222" style="3" customWidth="1"/>
+    <col min="45" max="45" width="18.5555555555556" style="3" customWidth="1"/>
     <col min="46" max="46" width="16.6666666666667" style="3" customWidth="1"/>
-    <col min="47" max="47" width="14.7809523809524" style="3" customWidth="1"/>
-    <col min="48" max="16384" width="8.88571428571429" style="3"/>
+    <col min="47" max="47" width="14.7777777777778" style="3" customWidth="1"/>
+    <col min="48" max="16384" width="8.88888888888889" style="3"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:47">
@@ -1757,7 +1757,7 @@
       <c r="AE1" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="9" t="s">
+      <c r="AF1" s="4" t="s">
         <v>31</v>
       </c>
       <c r="AG1" s="1" t="s">
@@ -1828,7 +1828,7 @@
       <c r="G2" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="H2" s="4" t="s">
+      <c r="H2" s="5" t="s">
         <v>52</v>
       </c>
       <c r="I2" s="2" t="s">
@@ -1949,7 +1949,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="3" s="3" customFormat="1" spans="1:37">
+    <row r="3" s="3" customFormat="1" spans="1:47">
       <c r="A3" s="1" t="s">
         <v>78</v>
       </c>
@@ -1974,7 +1974,7 @@
       <c r="H3" s="2" t="s">
         <v>80</v>
       </c>
-      <c r="I3" s="7" t="s">
+      <c r="I3" s="6" t="s">
         <v>81</v>
       </c>
       <c r="J3" s="2" t="s">
@@ -1992,7 +1992,7 @@
       <c r="N3" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="O3" s="8" t="s">
+      <c r="O3" s="7" t="s">
         <v>84</v>
       </c>
       <c r="P3" s="2" t="s">
@@ -2062,7 +2062,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="4" s="3" customFormat="1" spans="1:37">
+    <row r="4" s="3" customFormat="1" spans="1:47">
       <c r="A4" s="1" t="s">
         <v>87</v>
       </c>
@@ -2175,7 +2175,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="5" s="2" customFormat="1" customHeight="1" spans="1:37">
+    <row r="5" s="2" customFormat="1" ht="15" customHeight="1" spans="1:47">
       <c r="A5" s="1" t="s">
         <v>93</v>
       </c>
@@ -2188,13 +2188,13 @@
       <c r="D5" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="G5" s="8" t="s">
         <v>51</v>
       </c>
       <c r="H5" s="2" t="s">
@@ -2272,13 +2272,13 @@
       <c r="AF5" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="AG5" s="10" t="s">
+      <c r="AG5" s="9" t="s">
         <v>70</v>
       </c>
       <c r="AH5" s="11" t="s">
         <v>108</v>
       </c>
-      <c r="AI5" s="10" t="s">
+      <c r="AI5" s="9" t="s">
         <v>70</v>
       </c>
       <c r="AJ5" s="11" t="s">
@@ -2288,8 +2288,8 @@
         <v>55</v>
       </c>
     </row>
-    <row r="6" s="3" customFormat="1" ht="13" customHeight="1" spans="1:37">
-      <c r="A6" s="6" t="s">
+    <row r="6" s="3" customFormat="1" ht="13" customHeight="1" spans="1:47">
+      <c r="A6" s="10" t="s">
         <v>110</v>
       </c>
       <c r="B6" s="3" t="s">
@@ -2322,7 +2322,7 @@
       <c r="K6" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="L6" s="4" t="s">
+      <c r="L6" s="5" t="s">
         <v>112</v>
       </c>
       <c r="M6" s="2" t="s">
@@ -2385,13 +2385,13 @@
       <c r="AF6" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="AG6" s="10" t="s">
+      <c r="AG6" s="9" t="s">
         <v>118</v>
       </c>
       <c r="AH6" s="12" t="s">
         <v>119</v>
       </c>
-      <c r="AI6" s="10" t="s">
+      <c r="AI6" s="9" t="s">
         <v>70</v>
       </c>
       <c r="AJ6" s="12" t="s">
@@ -2401,8 +2401,8 @@
         <v>55</v>
       </c>
     </row>
-    <row r="7" s="3" customFormat="1" spans="1:37">
-      <c r="A7" s="6" t="s">
+    <row r="7" s="3" customFormat="1" spans="1:47">
+      <c r="A7" s="10" t="s">
         <v>121</v>
       </c>
       <c r="B7" s="3" t="s">
@@ -2435,7 +2435,7 @@
       <c r="K7" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="L7" s="4" t="s">
+      <c r="L7" s="5" t="s">
         <v>123</v>
       </c>
       <c r="M7" s="2" t="s">
@@ -2515,7 +2515,7 @@
       </c>
     </row>
     <row r="8" spans="1:47">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="10" t="s">
         <v>124</v>
       </c>
       <c r="B8" s="3" t="s">
@@ -2657,7 +2657,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="13" spans="11:11">
+    <row r="13" spans="1:47">
       <c r="K13" s="2"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
07.08.26 stabilizovani testovi placanja, i own account transfer
</commit_message>
<xml_diff>
--- a/testdata/data.xlsx
+++ b/testdata/data.xlsx
@@ -1,10 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000"/>
+    <workbookView windowWidth="23040" windowHeight="8340"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="127">
   <si>
     <t>username</t>
   </si>
@@ -333,6 +333,9 @@
   </si>
   <si>
     <t>205-9001033136870-28</t>
+  </si>
+  <si>
+    <t>RS35 2059 0310 3438 5543 96</t>
   </si>
   <si>
     <t>4313 **** **** 9452</t>
@@ -1037,7 +1040,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1067,6 +1070,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" quotePrefix="1">
       <alignment vertical="center"/>
@@ -1608,48 +1614,48 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:AW13"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="17.712962962963" customWidth="1"/>
-    <col min="2" max="2" width="33.5740740740741" customWidth="1"/>
-    <col min="4" max="6" width="22.1111111111111" customWidth="1"/>
+    <col min="1" max="1" width="17.7142857142857" customWidth="1"/>
+    <col min="2" max="2" width="33.5714285714286" customWidth="1"/>
+    <col min="4" max="6" width="22.1142857142857" customWidth="1"/>
     <col min="7" max="7" width="33" customWidth="1"/>
     <col min="8" max="8" width="23.6666666666667" customWidth="1"/>
-    <col min="9" max="10" width="33.8888888888889" customWidth="1"/>
+    <col min="9" max="10" width="33.8857142857143" customWidth="1"/>
     <col min="11" max="11" width="23.6666666666667" customWidth="1"/>
-    <col min="12" max="12" width="28.7407407407407" customWidth="1"/>
-    <col min="13" max="13" width="24.2222222222222" customWidth="1"/>
-    <col min="14" max="14" width="27.8888888888889" customWidth="1"/>
-    <col min="15" max="15" width="28.8611111111111" customWidth="1"/>
+    <col min="12" max="12" width="28.7428571428571" customWidth="1"/>
+    <col min="13" max="13" width="24.2190476190476" customWidth="1"/>
+    <col min="14" max="14" width="27.8857142857143" customWidth="1"/>
+    <col min="15" max="15" width="28.8571428571429" customWidth="1"/>
     <col min="16" max="16" width="26.6666666666667" customWidth="1"/>
     <col min="17" max="17" width="23.6666666666667" customWidth="1"/>
-    <col min="18" max="18" width="31.2222222222222" customWidth="1"/>
-    <col min="19" max="19" width="19.5555555555556" customWidth="1"/>
-    <col min="20" max="20" width="21.4444444444444" customWidth="1"/>
-    <col min="21" max="23" width="24.1111111111111" customWidth="1"/>
-    <col min="24" max="24" width="25.4259259259259" customWidth="1"/>
-    <col min="25" max="25" width="24.1111111111111" customWidth="1"/>
-    <col min="26" max="26" width="25.8796296296296" customWidth="1"/>
-    <col min="27" max="27" width="24.1111111111111" customWidth="1"/>
-    <col min="28" max="28" width="32.1851851851852" customWidth="1"/>
-    <col min="29" max="29" width="21.4444444444444" customWidth="1"/>
+    <col min="18" max="18" width="31.2190476190476" customWidth="1"/>
+    <col min="19" max="19" width="19.552380952381" customWidth="1"/>
+    <col min="20" max="20" width="21.447619047619" customWidth="1"/>
+    <col min="21" max="23" width="24.1142857142857" customWidth="1"/>
+    <col min="24" max="24" width="25.4285714285714" customWidth="1"/>
+    <col min="25" max="25" width="24.1142857142857" customWidth="1"/>
+    <col min="26" max="26" width="25.8761904761905" customWidth="1"/>
+    <col min="27" max="27" width="24.1142857142857" customWidth="1"/>
+    <col min="28" max="28" width="32.1809523809524" customWidth="1"/>
+    <col min="29" max="29" width="21.447619047619" customWidth="1"/>
     <col min="30" max="30" width="32.6666666666667" customWidth="1"/>
     <col min="31" max="31" width="17.6666666666667" customWidth="1"/>
-    <col min="32" max="32" width="23.8888888888889" customWidth="1"/>
-    <col min="33" max="33" width="26.0092592592593" customWidth="1"/>
-    <col min="34" max="34" width="23.5555555555556" customWidth="1"/>
-    <col min="35" max="35" width="26.0092592592593" customWidth="1"/>
-    <col min="36" max="36" width="23.5555555555556" customWidth="1"/>
-    <col min="37" max="37" width="23.7777777777778" customWidth="1"/>
+    <col min="32" max="32" width="23.8857142857143" customWidth="1"/>
+    <col min="33" max="33" width="26.0095238095238" customWidth="1"/>
+    <col min="34" max="34" width="23.552380952381" customWidth="1"/>
+    <col min="35" max="35" width="26.0095238095238" customWidth="1"/>
+    <col min="36" max="36" width="23.552380952381" customWidth="1"/>
+    <col min="37" max="37" width="23.7809523809524" customWidth="1"/>
     <col min="38" max="38" width="31" customWidth="1"/>
-    <col min="39" max="40" width="32.8888888888889" customWidth="1"/>
-    <col min="41" max="41" width="29.1111111111111" customWidth="1"/>
+    <col min="39" max="40" width="32.8857142857143" customWidth="1"/>
+    <col min="41" max="41" width="29.1142857142857" customWidth="1"/>
     <col min="42" max="42" width="33" customWidth="1"/>
-    <col min="43" max="43" width="37.1111111111111" customWidth="1"/>
-    <col min="44" max="44" width="31.2222222222222" customWidth="1"/>
-    <col min="45" max="45" width="18.5555555555556" customWidth="1"/>
+    <col min="43" max="43" width="37.1142857142857" customWidth="1"/>
+    <col min="44" max="44" width="31.2190476190476" customWidth="1"/>
+    <col min="45" max="45" width="18.552380952381" customWidth="1"/>
     <col min="46" max="46" width="16.6666666666667" customWidth="1"/>
-    <col min="47" max="47" width="14.7777777777778" customWidth="1"/>
+    <col min="47" max="47" width="14.7809523809524" customWidth="1"/>
     <col min="48" max="49" width="26.6666666666667" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1872,25 +1878,25 @@
       <c r="W2" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="X2" s="10" t="s">
+      <c r="X2" s="11" t="s">
         <v>66</v>
       </c>
       <c r="Y2" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="Z2" s="10" t="s">
+      <c r="Z2" s="11" t="s">
         <v>68</v>
       </c>
       <c r="AA2" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="AB2" s="10" t="s">
+      <c r="AB2" s="11" t="s">
         <v>70</v>
       </c>
       <c r="AC2" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="AD2" s="10" t="s">
+      <c r="AD2" s="11" t="s">
         <v>71</v>
       </c>
       <c r="AE2" s="2" t="s">
@@ -1902,7 +1908,7 @@
       <c r="AG2" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="AH2" s="10" t="s">
+      <c r="AH2" s="11" t="s">
         <v>73</v>
       </c>
       <c r="AI2" s="2" t="s">
@@ -2233,22 +2239,22 @@
         <v>101</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>54</v>
+        <v>102</v>
       </c>
       <c r="P5" s="2" t="s">
         <v>60</v>
       </c>
       <c r="Q5" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="R5" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="S5" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="T5" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="U5" s="2" t="s">
         <v>54</v>
@@ -2257,28 +2263,28 @@
         <v>54</v>
       </c>
       <c r="W5" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="X5" s="10" t="s">
         <v>107</v>
       </c>
+      <c r="X5" s="11" t="s">
+        <v>108</v>
+      </c>
       <c r="Y5" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="Z5" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
+      </c>
+      <c r="Z5" s="11" t="s">
+        <v>109</v>
       </c>
       <c r="AA5" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="AB5" s="10" t="s">
-        <v>109</v>
+      <c r="AB5" s="11" t="s">
+        <v>110</v>
       </c>
       <c r="AC5" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="AD5" s="10" t="s">
-        <v>110</v>
+      <c r="AD5" s="11" t="s">
+        <v>111</v>
       </c>
       <c r="AE5" s="2" t="s">
         <v>54</v>
@@ -2289,14 +2295,14 @@
       <c r="AG5" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="AH5" s="11" t="s">
-        <v>111</v>
+      <c r="AH5" s="12" t="s">
+        <v>112</v>
       </c>
       <c r="AI5" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="AJ5" s="11" t="s">
-        <v>111</v>
+      <c r="AJ5" s="12" t="s">
+        <v>112</v>
       </c>
       <c r="AK5" s="2" t="s">
         <v>57</v>
@@ -2305,7 +2311,7 @@
         <v>99</v>
       </c>
       <c r="AW5" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="6" s="3" customFormat="1" ht="13" customHeight="1" spans="1:49">
@@ -2352,22 +2358,22 @@
         <v>101</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>54</v>
+        <v>102</v>
       </c>
       <c r="P6" s="2" t="s">
         <v>60</v>
       </c>
       <c r="Q6" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="R6" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="S6" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="T6" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="U6" s="2" t="s">
         <v>54</v>
@@ -2376,28 +2382,28 @@
         <v>54</v>
       </c>
       <c r="W6" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="X6" s="10" t="s">
         <v>107</v>
       </c>
+      <c r="X6" s="11" t="s">
+        <v>108</v>
+      </c>
       <c r="Y6" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="Z6" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
+      </c>
+      <c r="Z6" s="11" t="s">
+        <v>109</v>
       </c>
       <c r="AA6" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="AB6" s="10" t="s">
-        <v>109</v>
+      <c r="AB6" s="11" t="s">
+        <v>110</v>
       </c>
       <c r="AC6" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="AD6" s="10" t="s">
-        <v>110</v>
+      <c r="AD6" s="11" t="s">
+        <v>111</v>
       </c>
       <c r="AE6" s="2" t="s">
         <v>54</v>
@@ -2408,14 +2414,14 @@
       <c r="AG6" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="AH6" s="11" t="s">
-        <v>111</v>
+      <c r="AH6" s="12" t="s">
+        <v>112</v>
       </c>
       <c r="AI6" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="AJ6" s="11" t="s">
-        <v>111</v>
+      <c r="AJ6" s="12" t="s">
+        <v>112</v>
       </c>
       <c r="AK6" s="2" t="s">
         <v>57</v>
@@ -2424,12 +2430,12 @@
         <v>99</v>
       </c>
       <c r="AW6" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="7" s="3" customFormat="1" spans="1:49">
       <c r="A7" s="8" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>54</v>
@@ -2450,7 +2456,7 @@
         <v>56</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>54</v>
@@ -2462,7 +2468,7 @@
         <v>54</v>
       </c>
       <c r="L7" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="M7" s="2" t="s">
         <v>54</v>
@@ -2548,7 +2554,7 @@
     </row>
     <row r="8" customFormat="1" spans="1:49">
       <c r="A8" s="8" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>54</v>
@@ -2602,10 +2608,10 @@
         <v>54</v>
       </c>
       <c r="S8" s="3" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="T8" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="U8" s="3" t="s">
         <v>54</v>
@@ -2697,7 +2703,7 @@
     </row>
     <row r="9" s="3" customFormat="1" ht="13" customHeight="1" spans="1:49">
       <c r="A9" s="8" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>54</v>
@@ -2718,7 +2724,7 @@
         <v>56</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>54</v>
@@ -2727,10 +2733,10 @@
         <v>53</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="L9" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="M9" s="2" t="s">
         <v>54</v>
@@ -2742,19 +2748,19 @@
         <v>54</v>
       </c>
       <c r="P9" s="2" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="R9" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="S9" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="T9" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="U9" s="2" t="s">
         <v>54</v>
@@ -2793,16 +2799,16 @@
         <v>54</v>
       </c>
       <c r="AG9" s="9" t="s">
-        <v>123</v>
-      </c>
-      <c r="AH9" s="11" t="s">
         <v>124</v>
+      </c>
+      <c r="AH9" s="12" t="s">
+        <v>125</v>
       </c>
       <c r="AI9" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="AJ9" s="11" t="s">
-        <v>125</v>
+      <c r="AJ9" s="12" t="s">
+        <v>126</v>
       </c>
       <c r="AK9" s="2" t="s">
         <v>57</v>
@@ -2815,12 +2821,12 @@
       </c>
     </row>
     <row r="10" spans="1:49">
-      <c r="AV10" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="AW10" s="2" t="s">
-        <v>54</v>
-      </c>
+      <c r="AR10" s="10"/>
+      <c r="AS10"/>
+      <c r="AT10"/>
+      <c r="AU10"/>
+      <c r="AV10" s="2"/>
+      <c r="AW10" s="2"/>
     </row>
     <row r="13" customFormat="1" spans="1:49">
       <c r="K13" s="2"/>

</xml_diff>